<commit_message>
Updated yamls with few shot examples
</commit_message>
<xml_diff>
--- a/data/few_shot/few_shot_dev.xlsx
+++ b/data/few_shot/few_shot_dev.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\panag\Desktop\ΙΕΛ ΕΡΓΑΣΙΑ\Εξετάσεις_γλωσσομάθειας\Πρότυπα_Πειραματικά\data\few_shot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8660114E-59A8-4BFA-B3E3-86CFDF1CA3E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAB7E6E2-957E-4FCA-AFC6-B9C2362523A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -482,9 +482,6 @@
 \nImplied Context: The presence of the nail, copper wire, and battery strongly suggests a basic physics setup for an electromagnet experiment, aimed at testing magnetic attraction.</t>
   </si>
   <si>
-    <t>['data\few_shot\electromagnet_experiment.png']</t>
-  </si>
-  <si>
     <t>Γνωρίζουμε ότι τα άλατα που συσσωρεύονται στα τοιχώματα ενός βραστήρα απομακρύνονται αν χρησιμοποιήσουμε λίγο ξίδι. Αν δεν υπάρχει διαθέσιμο ξίδι, ποια άλλα υλικά της καθημερινής ζωής θα μπορούσατε να χρησιμοποιήσετε για να καθαρίσετε τη συσκευή από τα άλατα;</t>
   </si>
   <si>
@@ -509,9 +506,6 @@
     <t>['DEV_MOCK_IMAGE_PHYSICS_CIRCUIT_SCHEMATIC.png', 'DEV_MOCK_IMAGE_PHYSICS_CIRCUIT_PHYSICAL.png']</t>
   </si>
   <si>
-    <t>['data\few_shot\electrical_circuit.png']</t>
-  </si>
-  <si>
     <t>multiple_choice</t>
   </si>
   <si>
@@ -615,9 +609,6 @@
   </si>
   <si>
     <t>ε1, α=35°, γ, β=45°, ε2</t>
-  </si>
-  <si>
-    <t>['data\few_shot\parallel_lines_and_angles.png']</t>
   </si>
   <si>
     <t>Αγοράσαμε 8 σακιά λιπάσματος για να ρίξουμε σε πέντε ίδια παρτέρια. Για να λιπάνουμε το ένα χρειάστηκε το $1\frac{1}{4}$ ενός σακιού. Πόσο λίπασμα θα περισσέψει αν λιπάνουμε και τα υπόλοιπα παρτέρια;</t>
@@ -651,9 +642,6 @@
     <t>The image shows a geometry problem involving nested triangles.\nTriangles: A large triangle $AB\Gamma$ ($ABC$) containing a smaller inner triangle $A\Delta E$ ($ADE$).\nBase Line: Points $B$, $\Delta$, $E$, and $\Gamma$ are collinear.\nMarkings:\nSides $AB$ and $A\Gamma$ have double tick marks, indicating $AB = A\Gamma$ (Triangle $AB\Gamma$ is isosceles).\nSides $A\Delta$ and $AE$ have single tick marks, indicating $A\Delta = AE$ (Triangle $A\Delta E$ is isosceles).\nAngles:\nAngle $\Gamma$ is labeled $50^{\circ}$.\nAngle $\Delta AE$ is labeled $50^{\circ}$.\nAngle $BA\Delta$ is labeled $x$.</t>
   </si>
   <si>
-    <t>['data\few_shot\geometry_diagram_angle.png']</t>
-  </si>
-  <si>
     <t>Η Μαρία στα διαγωνίσματα της Ιστορίας έχει πάρει τις εξής βαθμολογίες: 14, 17, 15, 16. Πόσο πρέπει να πάρει στο $5^{\circ}$ διαγώνισμα για να βγάλει μέσο όρο 16;</t>
   </si>
   <si>
@@ -727,6 +715,18 @@
   </si>
   <si>
     <t>['Α. επιβάλλεται με αυστηρότητα και στους υπόλοιπους ανθρώπους.', 'Β. συνδυάζεται με την πνευματική κάθαρση και την αποχή από τα πάθη.', 'Γ. αποσκοπεί αποκλειστικά στη βελτίωση της σωματικής μας υγείας.', 'Δ. τηρούνται κατά γράμμα μόνο οι διατροφικοί περιορισμοί.']</t>
+  </si>
+  <si>
+    <t>['data/few_shot/electromagnet_experiment.png']</t>
+  </si>
+  <si>
+    <t>['data/few_shot/electrical_circuit.png']</t>
+  </si>
+  <si>
+    <t>['data/few_shot/parallel_lines_and_angles.png']</t>
+  </si>
+  <si>
+    <t>['data/few_shot/geometry_diagram_angle.png']</t>
   </si>
 </sst>
 </file>
@@ -2094,7 +2094,7 @@
         <v>2.5</v>
       </c>
       <c r="R23" s="1" t="s">
-        <v>120</v>
+        <v>197</v>
       </c>
     </row>
     <row r="24" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
@@ -2111,13 +2111,13 @@
         <v>32</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>122</v>
       </c>
       <c r="N24" s="1">
         <v>2016</v>
@@ -2149,13 +2149,13 @@
         <v>32</v>
       </c>
       <c r="E25" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>124</v>
       </c>
       <c r="N25" s="1">
         <v>2017</v>
@@ -2187,19 +2187,19 @@
         <v>41</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I26" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="G26" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I26" s="1" t="s">
+      <c r="K26" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="N26" s="1">
         <v>2019</v>
@@ -2214,33 +2214,33 @@
         <v>3</v>
       </c>
       <c r="R26" s="1" t="s">
-        <v>129</v>
+        <v>198</v>
       </c>
     </row>
     <row r="27" spans="1:18" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="H27" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="I27" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>139</v>
       </c>
       <c r="J27" s="1">
         <v>1</v>
@@ -2266,28 +2266,28 @@
     </row>
     <row r="28" spans="1:18" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E28" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="H28" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="I28" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>143</v>
       </c>
       <c r="J28" s="1">
         <v>3</v>
@@ -2313,28 +2313,28 @@
     </row>
     <row r="29" spans="1:18" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E29" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="H29" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="I29" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>147</v>
       </c>
       <c r="J29" s="1">
         <v>1</v>
@@ -2360,28 +2360,28 @@
     </row>
     <row r="30" spans="1:18" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="H30" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="I30" s="1" t="s">
-        <v>151</v>
       </c>
       <c r="J30" s="1">
         <v>2</v>
@@ -2404,25 +2404,25 @@
     </row>
     <row r="31" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E31" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="I31" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="H31" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="J31" s="1">
         <v>4</v>
@@ -2448,37 +2448,37 @@
     </row>
     <row r="32" spans="1:18" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>86</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>41</v>
       </c>
       <c r="E32" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="H32" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="G32" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="I32" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J32" s="1">
         <v>1</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="M32" s="1">
         <v>2</v>
@@ -2496,30 +2496,30 @@
         <v>24</v>
       </c>
       <c r="R32" s="1" t="s">
-        <v>165</v>
+        <v>199</v>
       </c>
     </row>
     <row r="33" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>86</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J33" s="1">
         <v>3</v>
@@ -2542,25 +2542,25 @@
     </row>
     <row r="34" spans="1:18" ht="72" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>86</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J34" s="1">
         <v>3</v>
@@ -2583,34 +2583,34 @@
     </row>
     <row r="35" spans="1:18" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>86</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>41</v>
       </c>
       <c r="E35" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="I35" s="1" t="s">
         <v>170</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>173</v>
       </c>
       <c r="J35" s="1">
         <v>1</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="M35" s="1">
         <v>5</v>
@@ -2628,30 +2628,30 @@
         <v>3</v>
       </c>
       <c r="R35" s="1" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="36" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>86</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="J36" s="1">
         <v>2</v>
@@ -2677,28 +2677,28 @@
     </row>
     <row r="37" spans="1:18" ht="144" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="J37" s="1">
         <v>2</v>
@@ -2724,28 +2724,28 @@
     </row>
     <row r="38" spans="1:18" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J38" s="1">
         <v>3</v>
@@ -2771,28 +2771,28 @@
     </row>
     <row r="39" spans="1:18" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="J39" s="1">
         <v>0</v>
@@ -2818,28 +2818,28 @@
     </row>
     <row r="40" spans="1:18" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J40" s="1">
         <v>1</v>
@@ -2865,28 +2865,28 @@
     </row>
     <row r="41" spans="1:18" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J41" s="1">
         <v>1</v>

</xml_diff>